<commit_message>
Aktualisiere Datumsangaben in Sitemap und Metadaten; entferne .DS_Store
</commit_message>
<xml_diff>
--- a/docs/files/Excel-Vorlage-für-ISO-Toleranzen.xlsx
+++ b/docs/files/Excel-Vorlage-für-ISO-Toleranzen.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28627"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_50B48E0F4D524C66EDCE26D6A944B9B636854A00" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="105" windowWidth="18915" windowHeight="8505"/>
+    <workbookView xWindow="120" yWindow="105" windowWidth="18915" windowHeight="8505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -12,6 +13,11 @@
     <sheet name="Tabelle3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="125725"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -24,21 +30,60 @@
     <t>Welle</t>
   </si>
   <si>
+    <t>Toleranzlage</t>
+  </si>
+  <si>
+    <t>A - H</t>
+  </si>
+  <si>
+    <t>J - ZC</t>
+  </si>
+  <si>
+    <t>a - h</t>
+  </si>
+  <si>
+    <t>j - zc</t>
+  </si>
+  <si>
     <t>Passung</t>
   </si>
   <si>
+    <t>M6</t>
+  </si>
+  <si>
+    <t>k6</t>
+  </si>
+  <si>
     <t>Nennmaß</t>
   </si>
   <si>
+    <t>D =</t>
+  </si>
+  <si>
+    <t>d =</t>
+  </si>
+  <si>
     <t>Maßtoleranz</t>
   </si>
   <si>
     <t>oberes Abmaß</t>
   </si>
   <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>es</t>
+  </si>
+  <si>
     <t>unteres Abmaß</t>
   </si>
   <si>
+    <t>EI</t>
+  </si>
+  <si>
+    <t>ei</t>
+  </si>
+  <si>
     <t>Höchstmaß</t>
   </si>
   <si>
@@ -57,67 +102,28 @@
     <t>Höchstübermaß</t>
   </si>
   <si>
-    <t>ES</t>
-  </si>
-  <si>
-    <t>EI</t>
-  </si>
-  <si>
-    <t>es</t>
-  </si>
-  <si>
-    <t>ei</t>
-  </si>
-  <si>
-    <t>k6</t>
-  </si>
-  <si>
-    <t>D =</t>
-  </si>
-  <si>
-    <t>d =</t>
-  </si>
-  <si>
-    <t>j - zc</t>
-  </si>
-  <si>
-    <t>a - h</t>
-  </si>
-  <si>
-    <t>Toleranzlage</t>
-  </si>
-  <si>
-    <t>A - H</t>
-  </si>
-  <si>
-    <t>J - ZC</t>
+    <t>Art der Passung</t>
+  </si>
+  <si>
+    <t>Passtoleranz</t>
   </si>
   <si>
     <t>Hoch</t>
   </si>
   <si>
     <t>Tief</t>
-  </si>
-  <si>
-    <t>Passtoleranz</t>
-  </si>
-  <si>
-    <t>Art der Passung</t>
-  </si>
-  <si>
-    <t>M6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0\ &quot;µm&quot;"/>
     <numFmt numFmtId="165" formatCode="0\ &quot;mm&quot;"/>
-    <numFmt numFmtId="168" formatCode="#\ &quot;mm&quot;"/>
-    <numFmt numFmtId="171" formatCode="#.000\ &quot;mm&quot;"/>
-    <numFmt numFmtId="173" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="#\ &quot;mm&quot;"/>
+    <numFmt numFmtId="167" formatCode="#.000\ &quot;mm&quot;"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -298,71 +304,36 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="173" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="173" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -372,7 +343,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -380,11 +360,25 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -392,42 +386,45 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="173" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="168" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -442,13 +439,32 @@
       <color rgb="FFEEF3F8"/>
     </mruColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
   <c:lang val="de-DE"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <c:chart>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout>
         <c:manualLayout>
@@ -502,6 +518,12 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6F55-4BD9-9E50-00D7ECEF0B2F}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
@@ -543,7 +565,21 @@
               </c:numCache>
             </c:numRef>
           </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-6F55-4BD9-9E50-00D7ECEF0B2F}"/>
+            </c:ext>
+          </c:extLst>
         </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
         <c:hiLowLines>
           <c:spPr>
             <a:ln w="298450" cap="flat">
@@ -563,20 +599,25 @@
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="dd/mm/yyyy" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="120124160"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="120124160"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
+        <c:delete val="0"/>
         <c:axPos val="l"/>
         <c:majorGridlines>
           <c:spPr>
@@ -594,6 +635,8 @@
           </c:spPr>
         </c:majorGridlines>
         <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="120083584"/>
         <c:crosses val="autoZero"/>
@@ -604,6 +647,8 @@
       </c:spPr>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:ln>
@@ -635,7 +680,13 @@
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="5" name="Diagramm 4"/>
+        <xdr:cNvPr id="5" name="Diagramm 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000005000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
@@ -654,9 +705,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Larissa-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Larissa">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -694,7 +745,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Larissa">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -728,6 +779,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -762,9 +814,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Larissa">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -937,9 +990,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="5.7109375" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
@@ -952,446 +1005,453 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" thickBot="1">
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1" t="s">
+      <c r="D1" s="37"/>
+      <c r="E1" s="37" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1" t="s">
+      <c r="F1" s="37"/>
+      <c r="G1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1" t="s">
+      <c r="H1" s="37"/>
+      <c r="I1" s="37" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="1"/>
+      <c r="J1" s="37"/>
     </row>
     <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H2" s="3"/>
-      <c r="I2" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="J2" s="14"/>
+        <v>2</v>
+      </c>
+      <c r="C2" s="29" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="38"/>
+      <c r="G2" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="J2" s="38"/>
     </row>
     <row r="3" spans="1:10">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="35"/>
-      <c r="G3" s="33"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" s="35"/>
+        <v>7</v>
+      </c>
+      <c r="C3" s="26"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="28"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="27"/>
+      <c r="I3" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" s="28"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="31">
+        <v>10</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="23"/>
+      <c r="E4" s="20">
         <v>14</v>
       </c>
-      <c r="F4" s="32"/>
-      <c r="G4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="6"/>
-      <c r="I4" s="45">
+      <c r="F4" s="21"/>
+      <c r="G4" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="23"/>
+      <c r="I4" s="24">
         <v>14</v>
       </c>
-      <c r="J4" s="46"/>
+      <c r="J4" s="25"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="36">
+        <v>13</v>
+      </c>
+      <c r="C5" s="39">
         <v>11</v>
       </c>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="36">
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="41"/>
+      <c r="G5" s="39">
         <v>11</v>
       </c>
-      <c r="H5" s="37"/>
-      <c r="I5" s="37"/>
-      <c r="J5" s="38"/>
+      <c r="H5" s="40"/>
+      <c r="I5" s="40"/>
+      <c r="J5" s="41"/>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="18">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2">
         <f>D7+C5</f>
         <v>18</v>
       </c>
-      <c r="E6" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="39">
+      <c r="E6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="8">
         <v>-4</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="H6" s="40">
+      <c r="G6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="9">
         <v>34</v>
       </c>
-      <c r="I6" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="J6" s="10">
+      <c r="I6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="3">
         <f>J7+G5</f>
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="40">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="9">
         <v>7</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F7" s="19">
+      <c r="E7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="3">
         <f>F6-C5</f>
         <v>-15</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H7" s="8">
+      <c r="G7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="2">
         <f>H6-G5</f>
         <v>23</v>
       </c>
-      <c r="I7" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J7" s="39">
+      <c r="I7" t="s">
+        <v>19</v>
+      </c>
+      <c r="J7" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="17">
+        <v>20</v>
+      </c>
+      <c r="C8" s="34">
         <f>IF(E$3&gt;0,E$4+F6/1000,E$4+D6/1000)</f>
         <v>13.996</v>
       </c>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="17">
+      <c r="D8" s="35"/>
+      <c r="E8" s="35"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="34">
         <f>IF(I$3&gt;0,I$4+J6/1000,I$4+H6/1000)</f>
         <v>14.012</v>
       </c>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="16"/>
+      <c r="H8" s="35"/>
+      <c r="I8" s="35"/>
+      <c r="J8" s="36"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="17">
+        <v>21</v>
+      </c>
+      <c r="C9" s="34">
         <f>IF(E$3&gt;0,E$4+F7/1000,E$4+D7/1000)</f>
         <v>13.984999999999999</v>
       </c>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="17">
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="34">
         <f>IF(I$3&gt;0,I$4+J7/1000,I$4+H7/1000)</f>
         <v>14.000999999999999</v>
       </c>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="16"/>
+      <c r="H9" s="35"/>
+      <c r="I9" s="35"/>
+      <c r="J9" s="36"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="21">
+        <v>22</v>
+      </c>
+      <c r="C10" s="31">
         <f>C8-G9</f>
         <v>-4.9999999999990052E-3</v>
       </c>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="23"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="33"/>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="C11" s="21"/>
-      <c r="D11" s="22"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="22"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="23"/>
+        <v>23</v>
+      </c>
+      <c r="C11" s="31"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="33"/>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="C12" s="21">
+        <v>24</v>
+      </c>
+      <c r="C12" s="31">
         <f>C9-G8</f>
         <v>-2.7000000000001023E-2</v>
       </c>
-      <c r="D12" s="22"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="23"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="33"/>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" s="21"/>
-      <c r="D13" s="22"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="22"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="23"/>
+        <v>25</v>
+      </c>
+      <c r="C13" s="31"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="33"/>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>28</v>
-      </c>
-      <c r="C14" s="28" t="str">
+        <v>26</v>
+      </c>
+      <c r="C14" s="14" t="str">
         <f>IF(AND(C10&gt;0,C12&gt;0),"Spielpassung",IF(AND(C10&gt;0,C12&lt;0),"Übergangspassung",IF(AND(C10&lt;0,C12&lt;0),"Übermaßpassung","Fehler?")))</f>
         <v>Übermaßpassung</v>
       </c>
-      <c r="D14" s="29"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="29"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="30"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="16"/>
     </row>
     <row r="15" spans="1:10" ht="15.75" thickBot="1">
       <c r="A15" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="17">
         <f>C10-C12</f>
         <v>2.2000000000002018E-2</v>
       </c>
-      <c r="D15" s="11"/>
-      <c r="E15" s="11"/>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="12"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="19"/>
     </row>
     <row r="18" spans="1:9">
-      <c r="A18" s="24"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-      <c r="H18" s="24"/>
-    </row>
-    <row r="19" spans="1:9" s="26" customFormat="1">
-      <c r="A19" s="24"/>
-      <c r="B19" s="41"/>
-      <c r="C19" s="42" t="s">
-        <v>25</v>
-      </c>
-      <c r="D19" s="42" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19" s="27"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
-      <c r="I19" s="24"/>
-    </row>
-    <row r="20" spans="1:9" s="26" customFormat="1">
-      <c r="A20" s="24"/>
-      <c r="B20" s="43" t="str">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
+    </row>
+    <row r="19" spans="1:9" s="6" customFormat="1">
+      <c r="A19" s="4"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
+      <c r="I19" s="4"/>
+    </row>
+    <row r="20" spans="1:9" s="6" customFormat="1">
+      <c r="A20" s="4"/>
+      <c r="B20" s="12" t="str">
         <f>"Bohrung " &amp;E3&amp;C3</f>
         <v>Bohrung M6</v>
       </c>
-      <c r="C20" s="44">
+      <c r="C20" s="13">
         <f>C8</f>
         <v>13.996</v>
       </c>
-      <c r="D20" s="44">
+      <c r="D20" s="13">
         <f>C9</f>
         <v>13.984999999999999</v>
       </c>
-      <c r="E20" s="25"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
-      <c r="H20" s="24"/>
-      <c r="I20" s="24"/>
-    </row>
-    <row r="21" spans="1:9" s="26" customFormat="1">
-      <c r="A21" s="24"/>
-      <c r="B21" s="43" t="str">
+      <c r="E20" s="5"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
+      <c r="I20" s="4"/>
+    </row>
+    <row r="21" spans="1:9" s="6" customFormat="1">
+      <c r="A21" s="4"/>
+      <c r="B21" s="12" t="str">
         <f>"Welle " &amp;I3&amp;G3</f>
         <v>Welle k6</v>
       </c>
-      <c r="C21" s="44">
+      <c r="C21" s="13">
         <f>G8</f>
         <v>14.012</v>
       </c>
-      <c r="D21" s="44">
+      <c r="D21" s="13">
         <f>G9</f>
         <v>14.000999999999999</v>
       </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="24"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="24"/>
-      <c r="I21" s="24"/>
+      <c r="E21" s="5"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
+      <c r="I21" s="4"/>
     </row>
     <row r="22" spans="1:9">
-      <c r="A22" s="24"/>
-      <c r="B22" s="26"/>
-      <c r="C22" s="26"/>
-      <c r="D22" s="26"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="24"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="24"/>
-      <c r="I22" s="24"/>
+      <c r="A22" s="4"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
     </row>
     <row r="23" spans="1:9">
-      <c r="A23" s="24"/>
-      <c r="B23" s="24"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="24"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="24"/>
-      <c r="I23" s="24"/>
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
+      <c r="I23" s="4"/>
     </row>
     <row r="24" spans="1:9">
-      <c r="A24" s="24"/>
-      <c r="B24" s="24"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="24"/>
-      <c r="H24" s="24"/>
-      <c r="I24" s="24"/>
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
+      <c r="I24" s="4"/>
     </row>
     <row r="25" spans="1:9">
-      <c r="A25" s="24"/>
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
-      <c r="G25" s="24"/>
-      <c r="H25" s="24"/>
-      <c r="I25" s="24"/>
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
     </row>
     <row r="26" spans="1:9">
-      <c r="B26" s="24"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="24"/>
-      <c r="G26" s="24"/>
-      <c r="H26" s="24"/>
-      <c r="I26" s="24"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
+      <c r="I26" s="4"/>
     </row>
     <row r="27" spans="1:9">
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
     </row>
     <row r="28" spans="1:9">
-      <c r="B28" s="24"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="24"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="4"/>
     </row>
     <row r="29" spans="1:9">
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="4"/>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="26">
-    <mergeCell ref="C14:J14"/>
-    <mergeCell ref="C15:J15"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="I1:J1"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="E2:F2"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="I3:J3"/>
     <mergeCell ref="C2:D2"/>
@@ -1401,18 +1461,11 @@
     <mergeCell ref="G9:J9"/>
     <mergeCell ref="C9:F9"/>
     <mergeCell ref="C8:F8"/>
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="I1:J1"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="I2:J2"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="C1:D1"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="G2:H2"/>
-    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="C14:J14"/>
+    <mergeCell ref="C15:J15"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1421,18 +1474,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>